<commit_message>
xlwings_trial python scripts modified - random numbers and aging_buckets_parallel
</commit_message>
<xml_diff>
--- a/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
+++ b/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://0yt2k-my.sharepoint.com/personal/jignesh1567_0yt2k_onmicrosoft_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://0yt2k-my.sharepoint.com/personal/jignesh1567_0yt2k_onmicrosoft_com/Documents/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A71520D9-49BD-469C-9FFC-32ACF8CB9010}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FEF3F35-CA6D-476C-8390-27B0FDD823E5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B668F626-C124-440B-8D33-2C6D65FED1B1}"/>
   </bookViews>
@@ -61,9 +61,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.0000%"/>
+    <numFmt numFmtId="164" formatCode="0.0000%"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,6 +72,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -100,10 +108,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -439,16 +448,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10A0B8D4-FB59-41DD-9C12-088177A95D3A}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -465,49 +475,53 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>45343</v>
       </c>
       <c r="B2">
-        <v>536</v>
+        <v>1637</v>
       </c>
       <c r="C2" s="1">
         <v>43518</v>
       </c>
       <c r="D2">
-        <v>339</v>
+        <v>533</v>
       </c>
       <c r="E2" s="2">
         <f>(((B2/D2)^(1/(((A2-C2+1)/365)*4)))-1)*4</f>
-        <v>9.263296256233744E-2</v>
+        <v>0.23070477719433935</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E4">
         <f>A2-C2+1</f>
         <v>1826</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E5">
         <f>E4/365</f>
         <v>5.0027397260273974</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="E6">
         <f>E5*4</f>
         <v>20.010958904109589</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D7" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="3">
         <f>D2*((1+(E2/4))^E6)</f>
-        <v>535.99999999999977</v>
+        <v>1636.999999999998</v>
+      </c>
+      <c r="F7" s="3" t="b">
+        <f>E7=B2</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new tab in xlwings_trial for MAKEARRAY and co-pilot chat session
</commit_message>
<xml_diff>
--- a/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
+++ b/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://0yt2k-my.sharepoint.com/personal/jignesh1567_0yt2k_onmicrosoft_com/Documents/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FEF3F35-CA6D-476C-8390-27B0FDD823E5}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD212F29-294F-4171-A6F0-3CE4AD8170A8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B668F626-C124-440B-8D33-2C6D65FED1B1}"/>
   </bookViews>
@@ -33,6 +33,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -448,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10A0B8D4-FB59-41DD-9C12-088177A95D3A}">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
@@ -458,7 +480,7 @@
     <col min="5" max="5" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -475,53 +497,92 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>45343</v>
+        <v>45344</v>
       </c>
       <c r="B2">
-        <v>1637</v>
+        <v>376</v>
       </c>
       <c r="C2" s="1">
-        <v>43518</v>
+        <v>43525</v>
       </c>
       <c r="D2">
-        <v>533</v>
+        <v>67</v>
       </c>
       <c r="E2" s="2">
         <f>(((B2/D2)^(1/(((A2-C2+1)/365)*4)))-1)*4</f>
-        <v>0.23070477719433935</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>0.36132593061968077</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="J3" cm="1">
+        <f t="array" ref="J3:L6">_xlfn.MAKEARRAY(4,3,_xlfn.LAMBDA(_xlpm.r,_xlpm.c,_xlpm.r*_xlpm.c))</f>
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>2</v>
+      </c>
+      <c r="L3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E4">
         <f>A2-C2+1</f>
-        <v>1826</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1820</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>4</v>
+      </c>
+      <c r="L4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E5">
         <f>E4/365</f>
-        <v>5.0027397260273974</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>4.9863013698630141</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>6</v>
+      </c>
+      <c r="L5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E6">
         <f>E5*4</f>
-        <v>20.010958904109589</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>19.945205479452056</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+      <c r="K6">
+        <v>8</v>
+      </c>
+      <c r="L6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E7" s="3">
         <f>D2*((1+(E2/4))^E6)</f>
-        <v>1636.999999999998</v>
+        <v>375.99999999999937</v>
       </c>
       <c r="F7" s="3" t="b">
         <f>E7=B2</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Annualized Return Excel File Changed
</commit_message>
<xml_diff>
--- a/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
+++ b/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://0yt2k-my.sharepoint.com/personal/jignesh1567_0yt2k_onmicrosoft_com/Documents/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD212F29-294F-4171-A6F0-3CE4AD8170A8}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC3CECB3-C6D5-49BB-96E3-A7E4B82529F7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B668F626-C124-440B-8D33-2C6D65FED1B1}"/>
   </bookViews>
@@ -517,7 +517,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="J3" cm="1">
-        <f t="array" ref="J3:L6">_xlfn.MAKEARRAY(4,3,_xlfn.LAMBDA(_xlpm.r,_xlpm.c,_xlpm.r*_xlpm.c))</f>
+        <f t="array" ref="J3:L6">_xlfn.MAKEARRAY(4,3,_xlfn.LAMBDA(_xlpm.r,_xlpm.c,(_xlpm.r-1)*3+_xlpm.c))</f>
         <v>1</v>
       </c>
       <c r="K3">
@@ -533,10 +533,10 @@
         <v>1820</v>
       </c>
       <c r="J4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4">
         <v>6</v>
@@ -548,10 +548,10 @@
         <v>4.9863013698630141</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L5">
         <v>9</v>
@@ -563,10 +563,10 @@
         <v>19.945205479452056</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K6">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="L6">
         <v>12</v>

</xml_diff>

<commit_message>
Added recompiled dll using ucrt toolchain and changed downstream files
</commit_message>
<xml_diff>
--- a/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
+++ b/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/Derivation Annualized Return (Quarterly Compounded).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://0yt2k-my.sharepoint.com/personal/jignesh1567_0yt2k_onmicrosoft_com/Documents/Excel Examples Including  add-in xlwings and connected python - vba - dlls, etc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC3CECB3-C6D5-49BB-96E3-A7E4B82529F7}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="8_{2B178B50-43E2-41CB-B14B-28C0ED154751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B188D1F-E2CB-423F-8DFE-E47C2AA9ACFE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B668F626-C124-440B-8D33-2C6D65FED1B1}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Current Price</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>Check</t>
+  </si>
+  <si>
+    <t>Gold</t>
   </si>
 </sst>
 </file>
@@ -151,6 +154,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -499,20 +506,23 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>45344</v>
+        <v>45345</v>
       </c>
       <c r="B2">
-        <v>376</v>
+        <v>5380</v>
       </c>
       <c r="C2" s="1">
-        <v>43525</v>
+        <v>43524</v>
       </c>
       <c r="D2">
-        <v>67</v>
+        <v>2993</v>
       </c>
       <c r="E2" s="2">
         <f>(((B2/D2)^(1/(((A2-C2+1)/365)*4)))-1)*4</f>
-        <v>0.36132593061968077</v>
+        <v>0.11921761478412929</v>
+      </c>
+      <c r="F2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -530,7 +540,7 @@
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E4">
         <f>A2-C2+1</f>
-        <v>1820</v>
+        <v>1822</v>
       </c>
       <c r="J4">
         <v>4</v>
@@ -545,7 +555,7 @@
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E5">
         <f>E4/365</f>
-        <v>4.9863013698630141</v>
+        <v>4.9917808219178079</v>
       </c>
       <c r="J5">
         <v>7</v>
@@ -560,7 +570,7 @@
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E6">
         <f>E5*4</f>
-        <v>19.945205479452056</v>
+        <v>19.967123287671232</v>
       </c>
       <c r="J6">
         <v>10</v>
@@ -578,11 +588,11 @@
       </c>
       <c r="E7" s="3">
         <f>D2*((1+(E2/4))^E6)</f>
-        <v>375.99999999999937</v>
+        <v>5380.0000000000045</v>
       </c>
       <c r="F7" s="3" t="b">
         <f>E7=B2</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>